<commit_message>
feat: remove importacao CSV e mantem somente XLSX
</commit_message>
<xml_diff>
--- a/public/templates/contrato_gestao.xlsx
+++ b/public/templates/contrato_gestao.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orientacoes" sheetId="1" r:id="R086a9202bd444457"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ajuste" sheetId="2" r:id="R941b59e58cec4ffb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contratos" sheetId="3" r:id="R62c32854935548c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Naturezas_Contrato" sheetId="4" r:id="R4e760d5335c54852"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentos_Fiscais" sheetId="5" r:id="R543781b702944463"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pagamentos" sheetId="6" r:id="Rfe98f9c57b514a72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funcionarios" sheetId="7" r:id="R7b1abbb5b1b64980"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salarios" sheetId="8" r:id="Rdde81957495a4979"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remuneracoes_Func" sheetId="9" r:id="Ra72abfb9618746c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servidores_Cedidos" sheetId="10" r:id="Rd5de11c0a4954669"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remuneracoes_Cedidos" sheetId="11" r:id="R08d4e04bbe534f69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dicionario" sheetId="12" r:id="R193d1774571f410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orientacoes" sheetId="1" r:id="R1a8d951bbf7a4c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ajuste" sheetId="2" r:id="R9ccdfd4abe494bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contratos" sheetId="3" r:id="R5b2186eb60a343a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Naturezas_Contrato" sheetId="4" r:id="R30497094036047a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentos_Fiscais" sheetId="5" r:id="Rb57014170b09481d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pagamentos" sheetId="6" r:id="R4176d1a2cb134803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funcionarios" sheetId="7" r:id="R86dbc4c06bae4551"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salarios" sheetId="8" r:id="R75cc2264588d43fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remuneracoes_Func" sheetId="9" r:id="R847057263d004305"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servidores_Cedidos" sheetId="10" r:id="Rd400958828414423"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remuneracoes_Cedidos" sheetId="11" r:id="R08b3eb2fc17942a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dicionario" sheetId="12" r:id="Rf631dbef11a9478d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,10 +401,10 @@
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
       <x:c r="A11" s="1" t="str">
-        <x:v>CSV alternativo</x:v>
+        <x:v>Arquivo de carga</x:v>
       </x:c>
       <x:c r="B11" s="1" t="str">
-        <x:v>Um CSV UTF-8 por aba. Use o nome da aba como nome do arquivo. Ajuste.csv é obrigatório.</x:v>
+        <x:v>Envie somente um arquivo XLSX com todas as abas do ajuste.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="26" customHeight="1">

</xml_diff>